<commit_message>
feat: pointing bot updated
</commit_message>
<xml_diff>
--- a/04 - Pointing/01 - LP's/ApontamentoYesica.xlsx
+++ b/04 - Pointing/01 - LP's/ApontamentoYesica.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\feb3ct\Desktop\PyAutomateSAP\04 - Pointing\01 - LP's\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B258E588-4BDA-4FA5-86FA-26CA72321621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47E604B1-7151-4B56-A480-1BDB0156F6B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="94">
   <si>
     <t>LPs</t>
   </si>
@@ -302,6 +302,9 @@
   </si>
   <si>
     <t>LP053354</t>
+  </si>
+  <si>
+    <t>LP already have pointing!</t>
   </si>
 </sst>
 </file>
@@ -669,7 +672,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -684,55 +687,88 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
+      <c r="B2" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
+      <c r="B3" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
+      <c r="B4" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
+      <c r="B5" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
+      <c r="B6" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
+      <c r="B7" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
+      <c r="B8" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
+      <c r="B9" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
+      <c r="B10" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
+      <c r="B11" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>